<commit_message>
🔒 [FULL] Daily chip data 2026-06-05 22:53
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-06.xlsx
+++ b/data/reports/chip_radar_2026-06.xlsx
@@ -8065,10 +8065,10 @@
         </is>
       </c>
       <c r="E189" s="31" t="n">
-        <v>1776</v>
+        <v>1771</v>
       </c>
       <c r="F189" s="31" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G189" s="31" t="n">
         <v>23292</v>
@@ -8080,12 +8080,12 @@
         <v>21855</v>
       </c>
       <c r="J189" s="32" t="n">
-        <v>131.15</v>
+        <v>131.52</v>
       </c>
       <c r="K189" s="32" t="n">
-        <v>130.67</v>
-      </c>
-      <c r="L189" s="33">
+        <v>131.87</v>
+      </c>
+      <c r="L189" s="35">
         <f>F189*(K189-J189)</f>
         <v/>
       </c>
@@ -8135,10 +8135,10 @@
         </is>
       </c>
       <c r="E191" s="31" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F191" s="31" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G191" s="31" t="n">
         <v>5757</v>
@@ -8150,12 +8150,12 @@
         <v>4744</v>
       </c>
       <c r="J191" s="32" t="n">
-        <v>738.05</v>
+        <v>767.5700000000001</v>
       </c>
       <c r="K191" s="32" t="n">
-        <v>723.5</v>
-      </c>
-      <c r="L191" s="33">
+        <v>779.15</v>
+      </c>
+      <c r="L191" s="35">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -8170,10 +8170,10 @@
         </is>
       </c>
       <c r="E192" s="31" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F192" s="31" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G192" s="31" t="n">
         <v>4738</v>
@@ -8185,12 +8185,12 @@
         <v>2441</v>
       </c>
       <c r="J192" s="32" t="n">
-        <v>361.64</v>
+        <v>358.9</v>
       </c>
       <c r="K192" s="32" t="n">
-        <v>364.59</v>
-      </c>
-      <c r="L192" s="35">
+        <v>358.89</v>
+      </c>
+      <c r="L192" s="33">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -8205,7 +8205,7 @@
         </is>
       </c>
       <c r="E193" s="31" t="n">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="F193" s="31" t="n">
         <v>23</v>
@@ -8220,12 +8220,12 @@
         <v>3857</v>
       </c>
       <c r="J193" s="32" t="n">
-        <v>140.27</v>
+        <v>141.7</v>
       </c>
       <c r="K193" s="32" t="n">
         <v>140.39</v>
       </c>
-      <c r="L193" s="35">
+      <c r="L193" s="33">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -8306,29 +8306,29 @@
       <c r="C196" s="34" t="n"/>
       <c r="D196" s="30" t="inlineStr">
         <is>
-          <t>友達(2409)</t>
+          <t>大綜(3147)</t>
         </is>
       </c>
       <c r="E196" s="31" t="n">
-        <v>1046</v>
+        <v>106</v>
       </c>
       <c r="F196" s="31" t="n">
-        <v>943</v>
+        <v>0</v>
       </c>
       <c r="G196" s="31" t="n">
-        <v>2835</v>
+        <v>3016</v>
       </c>
       <c r="H196" s="31" t="n">
-        <v>2556</v>
+        <v>0</v>
       </c>
       <c r="I196" s="31" t="n">
-        <v>279</v>
+        <v>3016</v>
       </c>
       <c r="J196" s="32" t="n">
-        <v>27.1</v>
+        <v>284.5</v>
       </c>
       <c r="K196" s="32" t="n">
-        <v>27.1</v>
+        <v>0</v>
       </c>
       <c r="L196" s="35">
         <f>F196*(K196-J196)</f>
@@ -8376,31 +8376,31 @@
       <c r="C198" s="34" t="n"/>
       <c r="D198" s="30" t="inlineStr">
         <is>
-          <t>群創(3481)</t>
+          <t>華邦電(2344)</t>
         </is>
       </c>
       <c r="E198" s="31" t="n">
-        <v>442</v>
+        <v>158</v>
       </c>
       <c r="F198" s="31" t="n">
-        <v>320</v>
+        <v>47</v>
       </c>
       <c r="G198" s="31" t="n">
-        <v>2305</v>
+        <v>2560</v>
       </c>
       <c r="H198" s="31" t="n">
-        <v>1643</v>
+        <v>761</v>
       </c>
       <c r="I198" s="31" t="n">
-        <v>662</v>
+        <v>1799</v>
       </c>
       <c r="J198" s="32" t="n">
-        <v>52.15</v>
+        <v>162</v>
       </c>
       <c r="K198" s="32" t="n">
-        <v>51.35</v>
-      </c>
-      <c r="L198" s="33">
+        <v>162</v>
+      </c>
+      <c r="L198" s="35">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-06-06 00:25
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-06.xlsx
+++ b/data/reports/chip_radar_2026-06.xlsx
@@ -8065,10 +8065,10 @@
         </is>
       </c>
       <c r="E189" s="31" t="n">
-        <v>1771</v>
+        <v>1776</v>
       </c>
       <c r="F189" s="31" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G189" s="31" t="n">
         <v>23292</v>
@@ -8080,12 +8080,12 @@
         <v>21855</v>
       </c>
       <c r="J189" s="32" t="n">
-        <v>131.52</v>
+        <v>131.15</v>
       </c>
       <c r="K189" s="32" t="n">
-        <v>131.87</v>
-      </c>
-      <c r="L189" s="35">
+        <v>130.67</v>
+      </c>
+      <c r="L189" s="33">
         <f>F189*(K189-J189)</f>
         <v/>
       </c>
@@ -8135,10 +8135,10 @@
         </is>
       </c>
       <c r="E191" s="31" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F191" s="31" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G191" s="31" t="n">
         <v>5757</v>
@@ -8150,12 +8150,12 @@
         <v>4744</v>
       </c>
       <c r="J191" s="32" t="n">
-        <v>767.5700000000001</v>
+        <v>738.05</v>
       </c>
       <c r="K191" s="32" t="n">
-        <v>779.15</v>
-      </c>
-      <c r="L191" s="35">
+        <v>723.5</v>
+      </c>
+      <c r="L191" s="33">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -8170,10 +8170,10 @@
         </is>
       </c>
       <c r="E192" s="31" t="n">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F192" s="31" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G192" s="31" t="n">
         <v>4738</v>
@@ -8185,12 +8185,12 @@
         <v>2441</v>
       </c>
       <c r="J192" s="32" t="n">
-        <v>358.9</v>
+        <v>361.64</v>
       </c>
       <c r="K192" s="32" t="n">
-        <v>358.89</v>
-      </c>
-      <c r="L192" s="33">
+        <v>364.59</v>
+      </c>
+      <c r="L192" s="35">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -8205,7 +8205,7 @@
         </is>
       </c>
       <c r="E193" s="31" t="n">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="F193" s="31" t="n">
         <v>23</v>
@@ -8220,12 +8220,12 @@
         <v>3857</v>
       </c>
       <c r="J193" s="32" t="n">
-        <v>141.7</v>
+        <v>140.27</v>
       </c>
       <c r="K193" s="32" t="n">
         <v>140.39</v>
       </c>
-      <c r="L193" s="33">
+      <c r="L193" s="35">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -8306,29 +8306,29 @@
       <c r="C196" s="34" t="n"/>
       <c r="D196" s="30" t="inlineStr">
         <is>
-          <t>大綜(3147)</t>
+          <t>友達(2409)</t>
         </is>
       </c>
       <c r="E196" s="31" t="n">
-        <v>106</v>
+        <v>1046</v>
       </c>
       <c r="F196" s="31" t="n">
-        <v>0</v>
+        <v>943</v>
       </c>
       <c r="G196" s="31" t="n">
-        <v>3016</v>
+        <v>2835</v>
       </c>
       <c r="H196" s="31" t="n">
-        <v>0</v>
+        <v>2556</v>
       </c>
       <c r="I196" s="31" t="n">
-        <v>3016</v>
+        <v>279</v>
       </c>
       <c r="J196" s="32" t="n">
-        <v>284.5</v>
+        <v>27.1</v>
       </c>
       <c r="K196" s="32" t="n">
-        <v>0</v>
+        <v>27.1</v>
       </c>
       <c r="L196" s="35">
         <f>F196*(K196-J196)</f>
@@ -8376,31 +8376,31 @@
       <c r="C198" s="34" t="n"/>
       <c r="D198" s="30" t="inlineStr">
         <is>
-          <t>華邦電(2344)</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E198" s="31" t="n">
-        <v>158</v>
+        <v>442</v>
       </c>
       <c r="F198" s="31" t="n">
-        <v>47</v>
+        <v>320</v>
       </c>
       <c r="G198" s="31" t="n">
-        <v>2560</v>
+        <v>2305</v>
       </c>
       <c r="H198" s="31" t="n">
-        <v>761</v>
+        <v>1643</v>
       </c>
       <c r="I198" s="31" t="n">
-        <v>1799</v>
+        <v>662</v>
       </c>
       <c r="J198" s="32" t="n">
-        <v>162</v>
+        <v>52.15</v>
       </c>
       <c r="K198" s="32" t="n">
-        <v>162</v>
-      </c>
-      <c r="L198" s="35">
+        <v>51.35</v>
+      </c>
+      <c r="L198" s="33">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-06-06 01:16
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-06.xlsx
+++ b/data/reports/chip_radar_2026-06.xlsx
@@ -8065,10 +8065,10 @@
         </is>
       </c>
       <c r="E189" s="31" t="n">
-        <v>1776</v>
+        <v>1771</v>
       </c>
       <c r="F189" s="31" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G189" s="31" t="n">
         <v>23292</v>
@@ -8080,12 +8080,12 @@
         <v>21855</v>
       </c>
       <c r="J189" s="32" t="n">
-        <v>131.15</v>
+        <v>131.52</v>
       </c>
       <c r="K189" s="32" t="n">
-        <v>130.67</v>
-      </c>
-      <c r="L189" s="33">
+        <v>131.87</v>
+      </c>
+      <c r="L189" s="35">
         <f>F189*(K189-J189)</f>
         <v/>
       </c>
@@ -8135,10 +8135,10 @@
         </is>
       </c>
       <c r="E191" s="31" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F191" s="31" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G191" s="31" t="n">
         <v>5757</v>
@@ -8150,12 +8150,12 @@
         <v>4744</v>
       </c>
       <c r="J191" s="32" t="n">
-        <v>738.05</v>
+        <v>767.5700000000001</v>
       </c>
       <c r="K191" s="32" t="n">
-        <v>723.5</v>
-      </c>
-      <c r="L191" s="33">
+        <v>779.15</v>
+      </c>
+      <c r="L191" s="35">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -8170,10 +8170,10 @@
         </is>
       </c>
       <c r="E192" s="31" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F192" s="31" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G192" s="31" t="n">
         <v>4738</v>
@@ -8185,12 +8185,12 @@
         <v>2441</v>
       </c>
       <c r="J192" s="32" t="n">
-        <v>361.64</v>
+        <v>358.9</v>
       </c>
       <c r="K192" s="32" t="n">
-        <v>364.59</v>
-      </c>
-      <c r="L192" s="35">
+        <v>358.89</v>
+      </c>
+      <c r="L192" s="33">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -8205,7 +8205,7 @@
         </is>
       </c>
       <c r="E193" s="31" t="n">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="F193" s="31" t="n">
         <v>23</v>
@@ -8220,12 +8220,12 @@
         <v>3857</v>
       </c>
       <c r="J193" s="32" t="n">
-        <v>140.27</v>
+        <v>141.7</v>
       </c>
       <c r="K193" s="32" t="n">
         <v>140.39</v>
       </c>
-      <c r="L193" s="35">
+      <c r="L193" s="33">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -8306,29 +8306,29 @@
       <c r="C196" s="34" t="n"/>
       <c r="D196" s="30" t="inlineStr">
         <is>
-          <t>友達(2409)</t>
+          <t>大綜(3147)</t>
         </is>
       </c>
       <c r="E196" s="31" t="n">
-        <v>1046</v>
+        <v>106</v>
       </c>
       <c r="F196" s="31" t="n">
-        <v>943</v>
+        <v>0</v>
       </c>
       <c r="G196" s="31" t="n">
-        <v>2835</v>
+        <v>3016</v>
       </c>
       <c r="H196" s="31" t="n">
-        <v>2556</v>
+        <v>0</v>
       </c>
       <c r="I196" s="31" t="n">
-        <v>279</v>
+        <v>3016</v>
       </c>
       <c r="J196" s="32" t="n">
-        <v>27.1</v>
+        <v>284.5</v>
       </c>
       <c r="K196" s="32" t="n">
-        <v>27.1</v>
+        <v>0</v>
       </c>
       <c r="L196" s="35">
         <f>F196*(K196-J196)</f>
@@ -8376,31 +8376,31 @@
       <c r="C198" s="34" t="n"/>
       <c r="D198" s="30" t="inlineStr">
         <is>
-          <t>群創(3481)</t>
+          <t>華邦電(2344)</t>
         </is>
       </c>
       <c r="E198" s="31" t="n">
-        <v>442</v>
+        <v>158</v>
       </c>
       <c r="F198" s="31" t="n">
-        <v>320</v>
+        <v>47</v>
       </c>
       <c r="G198" s="31" t="n">
-        <v>2305</v>
+        <v>2560</v>
       </c>
       <c r="H198" s="31" t="n">
-        <v>1643</v>
+        <v>761</v>
       </c>
       <c r="I198" s="31" t="n">
-        <v>662</v>
+        <v>1799</v>
       </c>
       <c r="J198" s="32" t="n">
-        <v>52.15</v>
+        <v>162</v>
       </c>
       <c r="K198" s="32" t="n">
-        <v>51.35</v>
-      </c>
-      <c r="L198" s="33">
+        <v>162</v>
+      </c>
+      <c r="L198" s="35">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-06-06 13:34
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-06.xlsx
+++ b/data/reports/chip_radar_2026-06.xlsx
@@ -8065,10 +8065,10 @@
         </is>
       </c>
       <c r="E189" s="31" t="n">
-        <v>1771</v>
+        <v>1776</v>
       </c>
       <c r="F189" s="31" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G189" s="31" t="n">
         <v>23292</v>
@@ -8080,12 +8080,12 @@
         <v>21855</v>
       </c>
       <c r="J189" s="32" t="n">
-        <v>131.52</v>
+        <v>131.15</v>
       </c>
       <c r="K189" s="32" t="n">
-        <v>131.87</v>
-      </c>
-      <c r="L189" s="35">
+        <v>130.67</v>
+      </c>
+      <c r="L189" s="33">
         <f>F189*(K189-J189)</f>
         <v/>
       </c>
@@ -8135,10 +8135,10 @@
         </is>
       </c>
       <c r="E191" s="31" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F191" s="31" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G191" s="31" t="n">
         <v>5757</v>
@@ -8150,12 +8150,12 @@
         <v>4744</v>
       </c>
       <c r="J191" s="32" t="n">
-        <v>767.5700000000001</v>
+        <v>738.05</v>
       </c>
       <c r="K191" s="32" t="n">
-        <v>779.15</v>
-      </c>
-      <c r="L191" s="35">
+        <v>723.5</v>
+      </c>
+      <c r="L191" s="33">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -8170,10 +8170,10 @@
         </is>
       </c>
       <c r="E192" s="31" t="n">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F192" s="31" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G192" s="31" t="n">
         <v>4738</v>
@@ -8185,12 +8185,12 @@
         <v>2441</v>
       </c>
       <c r="J192" s="32" t="n">
-        <v>358.9</v>
+        <v>361.64</v>
       </c>
       <c r="K192" s="32" t="n">
-        <v>358.89</v>
-      </c>
-      <c r="L192" s="33">
+        <v>364.59</v>
+      </c>
+      <c r="L192" s="35">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -8205,7 +8205,7 @@
         </is>
       </c>
       <c r="E193" s="31" t="n">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="F193" s="31" t="n">
         <v>23</v>
@@ -8220,12 +8220,12 @@
         <v>3857</v>
       </c>
       <c r="J193" s="32" t="n">
-        <v>141.7</v>
+        <v>140.27</v>
       </c>
       <c r="K193" s="32" t="n">
         <v>140.39</v>
       </c>
-      <c r="L193" s="33">
+      <c r="L193" s="35">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -8306,29 +8306,29 @@
       <c r="C196" s="34" t="n"/>
       <c r="D196" s="30" t="inlineStr">
         <is>
-          <t>大綜(3147)</t>
+          <t>友達(2409)</t>
         </is>
       </c>
       <c r="E196" s="31" t="n">
-        <v>106</v>
+        <v>1046</v>
       </c>
       <c r="F196" s="31" t="n">
-        <v>0</v>
+        <v>943</v>
       </c>
       <c r="G196" s="31" t="n">
-        <v>3016</v>
+        <v>2835</v>
       </c>
       <c r="H196" s="31" t="n">
-        <v>0</v>
+        <v>2556</v>
       </c>
       <c r="I196" s="31" t="n">
-        <v>3016</v>
+        <v>279</v>
       </c>
       <c r="J196" s="32" t="n">
-        <v>284.5</v>
+        <v>27.1</v>
       </c>
       <c r="K196" s="32" t="n">
-        <v>0</v>
+        <v>27.1</v>
       </c>
       <c r="L196" s="35">
         <f>F196*(K196-J196)</f>
@@ -8376,31 +8376,31 @@
       <c r="C198" s="34" t="n"/>
       <c r="D198" s="30" t="inlineStr">
         <is>
-          <t>華邦電(2344)</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E198" s="31" t="n">
-        <v>158</v>
+        <v>442</v>
       </c>
       <c r="F198" s="31" t="n">
-        <v>47</v>
+        <v>320</v>
       </c>
       <c r="G198" s="31" t="n">
-        <v>2560</v>
+        <v>2305</v>
       </c>
       <c r="H198" s="31" t="n">
-        <v>761</v>
+        <v>1643</v>
       </c>
       <c r="I198" s="31" t="n">
-        <v>1799</v>
+        <v>662</v>
       </c>
       <c r="J198" s="32" t="n">
-        <v>162</v>
+        <v>52.15</v>
       </c>
       <c r="K198" s="32" t="n">
-        <v>162</v>
-      </c>
-      <c r="L198" s="35">
+        <v>51.35</v>
+      </c>
+      <c r="L198" s="33">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>
@@ -16507,29 +16507,29 @@
       <c r="C411" s="95" t="n"/>
       <c r="D411" s="91" t="inlineStr">
         <is>
-          <t>光聖(6442)</t>
+          <t>波若威(3163)</t>
         </is>
       </c>
       <c r="E411" s="92" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F411" s="92" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="G411" s="92" t="n">
-        <v>5294</v>
+        <v>2487</v>
       </c>
       <c r="H411" s="92" t="n">
-        <v>2768</v>
+        <v>236</v>
       </c>
       <c r="I411" s="92" t="n">
-        <v>2526</v>
+        <v>2251</v>
       </c>
       <c r="J411" s="93" t="n">
-        <v>2036.27</v>
+        <v>1036.29</v>
       </c>
       <c r="K411" s="93" t="n">
-        <v>2129.23</v>
+        <v>1182</v>
       </c>
       <c r="L411" s="96">
         <f>F411*(K411-J411)</f>
@@ -16542,31 +16542,31 @@
       <c r="C412" s="95" t="n"/>
       <c r="D412" s="91" t="inlineStr">
         <is>
-          <t>上詮(3363)</t>
+          <t>聖暉*(5536)</t>
         </is>
       </c>
       <c r="E412" s="92" t="n">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="F412" s="92" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="G412" s="92" t="n">
-        <v>4271</v>
+        <v>1607</v>
       </c>
       <c r="H412" s="92" t="n">
-        <v>2135</v>
+        <v>621</v>
       </c>
       <c r="I412" s="92" t="n">
-        <v>2136</v>
+        <v>986</v>
       </c>
       <c r="J412" s="93" t="n">
-        <v>908.72</v>
+        <v>1147.71</v>
       </c>
       <c r="K412" s="93" t="n">
-        <v>889.67</v>
-      </c>
-      <c r="L412" s="94">
+        <v>1241.8</v>
+      </c>
+      <c r="L412" s="96">
         <f>F412*(K412-J412)</f>
         <v/>
       </c>
@@ -16577,31 +16577,31 @@
       <c r="C413" s="95" t="n"/>
       <c r="D413" s="91" t="inlineStr">
         <is>
-          <t>台新新光金(2887)</t>
+          <t>佳必琪(6197)</t>
         </is>
       </c>
       <c r="E413" s="92" t="n">
-        <v>1179</v>
+        <v>36</v>
       </c>
       <c r="F413" s="92" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="G413" s="92" t="n">
-        <v>3310</v>
+        <v>1184</v>
       </c>
       <c r="H413" s="92" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I413" s="92" t="n">
-        <v>3250</v>
+        <v>1120</v>
       </c>
       <c r="J413" s="93" t="n">
-        <v>28.08</v>
+        <v>329</v>
       </c>
       <c r="K413" s="93" t="n">
-        <v>28.38</v>
-      </c>
-      <c r="L413" s="96">
+        <v>322.5</v>
+      </c>
+      <c r="L413" s="94">
         <f>F413*(K413-J413)</f>
         <v/>
       </c>
@@ -16612,29 +16612,29 @@
       <c r="C414" s="95" t="n"/>
       <c r="D414" s="91" t="inlineStr">
         <is>
-          <t>聖暉*(5536)</t>
+          <t>遠雄(5522)</t>
         </is>
       </c>
       <c r="E414" s="92" t="n">
-        <v>14</v>
+        <v>114</v>
       </c>
       <c r="F414" s="92" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G414" s="92" t="n">
-        <v>1607</v>
+        <v>869</v>
       </c>
       <c r="H414" s="92" t="n">
-        <v>621</v>
+        <v>0</v>
       </c>
       <c r="I414" s="92" t="n">
-        <v>986</v>
+        <v>869</v>
       </c>
       <c r="J414" s="93" t="n">
-        <v>1147.71</v>
+        <v>76.25</v>
       </c>
       <c r="K414" s="93" t="n">
-        <v>1241.8</v>
+        <v>0</v>
       </c>
       <c r="L414" s="96">
         <f>F414*(K414-J414)</f>
@@ -16647,31 +16647,31 @@
       <c r="C415" s="95" t="n"/>
       <c r="D415" s="91" t="inlineStr">
         <is>
-          <t>可成(2474)</t>
+          <t>兆利(3548)</t>
         </is>
       </c>
       <c r="E415" s="92" t="n">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="F415" s="92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G415" s="92" t="n">
-        <v>1185</v>
+        <v>637</v>
       </c>
       <c r="H415" s="92" t="n">
-        <v>93</v>
+        <v>31</v>
       </c>
       <c r="I415" s="92" t="n">
-        <v>1092</v>
+        <v>606</v>
       </c>
       <c r="J415" s="93" t="n">
-        <v>232.35</v>
+        <v>104.49</v>
       </c>
       <c r="K415" s="93" t="n">
-        <v>231.5</v>
-      </c>
-      <c r="L415" s="94">
+        <v>104.67</v>
+      </c>
+      <c r="L415" s="96">
         <f>F415*(K415-J415)</f>
         <v/>
       </c>
@@ -16682,29 +16682,29 @@
       <c r="C416" s="95" t="n"/>
       <c r="D416" s="91" t="inlineStr">
         <is>
-          <t>川湖(2059)</t>
+          <t>華盈(3520)</t>
         </is>
       </c>
       <c r="E416" s="92" t="n">
-        <v>2</v>
+        <v>163</v>
       </c>
       <c r="F416" s="92" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G416" s="92" t="n">
-        <v>1139</v>
+        <v>278</v>
       </c>
       <c r="H416" s="92" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I416" s="92" t="n">
-        <v>1133</v>
+        <v>270</v>
       </c>
       <c r="J416" s="93" t="n">
-        <v>5695</v>
+        <v>17.05</v>
       </c>
       <c r="K416" s="93" t="n">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="L416" s="94">
         <f>F416*(K416-J416)</f>
@@ -16715,71 +16715,33 @@
       <c r="A417" s="95" t="n"/>
       <c r="B417" s="95" t="n"/>
       <c r="C417" s="95" t="n"/>
-      <c r="D417" s="91" t="inlineStr">
-        <is>
-          <t>長華*(8070)</t>
-        </is>
-      </c>
-      <c r="E417" s="92" t="n">
-        <v>179</v>
-      </c>
-      <c r="F417" s="92" t="n">
-        <v>5</v>
-      </c>
-      <c r="G417" s="92" t="n">
-        <v>1121</v>
-      </c>
-      <c r="H417" s="92" t="n">
-        <v>32</v>
-      </c>
-      <c r="I417" s="92" t="n">
-        <v>1089</v>
-      </c>
-      <c r="J417" s="93" t="n">
-        <v>62.61</v>
-      </c>
-      <c r="K417" s="93" t="n">
-        <v>64.2</v>
-      </c>
-      <c r="L417" s="96">
-        <f>F417*(K417-J417)</f>
-        <v/>
-      </c>
+      <c r="D417" s="98" t="inlineStr">
+        <is>
+          <t>⚪ 今日漲停僅 8 檔</t>
+        </is>
+      </c>
+      <c r="E417" s="92" t="n"/>
+      <c r="F417" s="92" t="n"/>
+      <c r="G417" s="92" t="n"/>
+      <c r="H417" s="92" t="n"/>
+      <c r="I417" s="92" t="n"/>
+      <c r="J417" s="93" t="n"/>
+      <c r="K417" s="93" t="n"/>
+      <c r="L417" s="96" t="n"/>
     </row>
     <row r="418" ht="16.5" customHeight="1">
       <c r="A418" s="95" t="n"/>
       <c r="B418" s="95" t="n"/>
       <c r="C418" s="95" t="n"/>
-      <c r="D418" s="91" t="inlineStr">
-        <is>
-          <t>兆利(3548)</t>
-        </is>
-      </c>
-      <c r="E418" s="92" t="n">
-        <v>61</v>
-      </c>
-      <c r="F418" s="92" t="n">
-        <v>3</v>
-      </c>
-      <c r="G418" s="92" t="n">
-        <v>637</v>
-      </c>
-      <c r="H418" s="92" t="n">
-        <v>31</v>
-      </c>
-      <c r="I418" s="92" t="n">
-        <v>606</v>
-      </c>
-      <c r="J418" s="93" t="n">
-        <v>104.49</v>
-      </c>
-      <c r="K418" s="93" t="n">
-        <v>104.67</v>
-      </c>
-      <c r="L418" s="96">
-        <f>F418*(K418-J418)</f>
-        <v/>
-      </c>
+      <c r="D418" s="91" t="n"/>
+      <c r="E418" s="92" t="n"/>
+      <c r="F418" s="92" t="n"/>
+      <c r="G418" s="92" t="n"/>
+      <c r="H418" s="92" t="n"/>
+      <c r="I418" s="92" t="n"/>
+      <c r="J418" s="93" t="n"/>
+      <c r="K418" s="93" t="n"/>
+      <c r="L418" s="96" t="n"/>
     </row>
     <row r="419" ht="16.5" customHeight="1">
       <c r="A419" s="97" t="n"/>
@@ -16853,31 +16815,31 @@
       </c>
       <c r="D420" s="91" t="inlineStr">
         <is>
-          <t>訊芯-KY(6451)</t>
+          <t>科嶠(4542)</t>
         </is>
       </c>
       <c r="E420" s="92" t="n">
-        <v>69</v>
+        <v>137</v>
       </c>
       <c r="F420" s="92" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="G420" s="92" t="n">
-        <v>4736</v>
+        <v>3768</v>
       </c>
       <c r="H420" s="92" t="n">
-        <v>1103</v>
+        <v>179</v>
       </c>
       <c r="I420" s="92" t="n">
-        <v>3633</v>
+        <v>3589</v>
       </c>
       <c r="J420" s="93" t="n">
-        <v>686.38</v>
+        <v>275.05</v>
       </c>
       <c r="K420" s="93" t="n">
-        <v>689.62</v>
-      </c>
-      <c r="L420" s="96">
+        <v>255.86</v>
+      </c>
+      <c r="L420" s="94">
         <f>F420*(K420-J420)</f>
         <v/>
       </c>
@@ -16888,31 +16850,31 @@
       <c r="C421" s="95" t="n"/>
       <c r="D421" s="91" t="inlineStr">
         <is>
-          <t>川湖(2059)</t>
+          <t>金居(8358)</t>
         </is>
       </c>
       <c r="E421" s="92" t="n">
+        <v>22</v>
+      </c>
+      <c r="F421" s="92" t="n">
         <v>7</v>
       </c>
-      <c r="F421" s="92" t="n">
-        <v>1</v>
-      </c>
       <c r="G421" s="92" t="n">
-        <v>3773</v>
+        <v>1332</v>
       </c>
       <c r="H421" s="92" t="n">
-        <v>73</v>
+        <v>434</v>
       </c>
       <c r="I421" s="92" t="n">
-        <v>3700</v>
+        <v>898</v>
       </c>
       <c r="J421" s="93" t="n">
-        <v>5389.57</v>
+        <v>605.5</v>
       </c>
       <c r="K421" s="93" t="n">
-        <v>730</v>
-      </c>
-      <c r="L421" s="94">
+        <v>620</v>
+      </c>
+      <c r="L421" s="96">
         <f>F421*(K421-J421)</f>
         <v/>
       </c>
@@ -16923,31 +16885,31 @@
       <c r="C422" s="95" t="n"/>
       <c r="D422" s="91" t="inlineStr">
         <is>
-          <t>上詮(3363)</t>
+          <t>佳必琪(6197)</t>
         </is>
       </c>
       <c r="E422" s="92" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="F422" s="92" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G422" s="92" t="n">
-        <v>2580</v>
+        <v>1298</v>
       </c>
       <c r="H422" s="92" t="n">
-        <v>892</v>
+        <v>198</v>
       </c>
       <c r="I422" s="92" t="n">
-        <v>1688</v>
+        <v>1100</v>
       </c>
       <c r="J422" s="93" t="n">
-        <v>921.3200000000001</v>
+        <v>324.6</v>
       </c>
       <c r="K422" s="93" t="n">
-        <v>892</v>
-      </c>
-      <c r="L422" s="94">
+        <v>329.83</v>
+      </c>
+      <c r="L422" s="96">
         <f>F422*(K422-J422)</f>
         <v/>
       </c>
@@ -16991,211 +16953,89 @@
       <c r="A424" s="95" t="n"/>
       <c r="B424" s="95" t="n"/>
       <c r="C424" s="95" t="n"/>
-      <c r="D424" s="91" t="inlineStr">
-        <is>
-          <t>友達(2409)</t>
-        </is>
-      </c>
-      <c r="E424" s="92" t="n">
-        <v>364</v>
-      </c>
-      <c r="F424" s="92" t="n">
-        <v>237</v>
-      </c>
-      <c r="G424" s="92" t="n">
-        <v>986</v>
-      </c>
-      <c r="H424" s="92" t="n">
-        <v>642</v>
-      </c>
-      <c r="I424" s="92" t="n">
-        <v>344</v>
-      </c>
-      <c r="J424" s="93" t="n">
-        <v>27.1</v>
-      </c>
-      <c r="K424" s="93" t="n">
-        <v>27.1</v>
-      </c>
-      <c r="L424" s="96">
-        <f>F424*(K424-J424)</f>
-        <v/>
-      </c>
+      <c r="D424" s="98" t="inlineStr">
+        <is>
+          <t>⚪ 今日漲停僅 4 檔</t>
+        </is>
+      </c>
+      <c r="E424" s="92" t="n"/>
+      <c r="F424" s="92" t="n"/>
+      <c r="G424" s="92" t="n"/>
+      <c r="H424" s="92" t="n"/>
+      <c r="I424" s="92" t="n"/>
+      <c r="J424" s="93" t="n"/>
+      <c r="K424" s="93" t="n"/>
+      <c r="L424" s="96" t="n"/>
     </row>
     <row r="425" ht="16.5" customHeight="1">
       <c r="A425" s="95" t="n"/>
       <c r="B425" s="95" t="n"/>
       <c r="C425" s="95" t="n"/>
-      <c r="D425" s="91" t="inlineStr">
-        <is>
-          <t>創新服務(7828)</t>
-        </is>
-      </c>
-      <c r="E425" s="92" t="n">
-        <v>6</v>
-      </c>
-      <c r="F425" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G425" s="92" t="n">
-        <v>962</v>
-      </c>
-      <c r="H425" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="I425" s="92" t="n">
-        <v>962</v>
-      </c>
-      <c r="J425" s="93" t="n">
-        <v>1603.83</v>
-      </c>
-      <c r="K425" s="93" t="n">
-        <v>0</v>
-      </c>
-      <c r="L425" s="96">
-        <f>F425*(K425-J425)</f>
-        <v/>
-      </c>
+      <c r="D425" s="91" t="n"/>
+      <c r="E425" s="92" t="n"/>
+      <c r="F425" s="92" t="n"/>
+      <c r="G425" s="92" t="n"/>
+      <c r="H425" s="92" t="n"/>
+      <c r="I425" s="92" t="n"/>
+      <c r="J425" s="93" t="n"/>
+      <c r="K425" s="93" t="n"/>
+      <c r="L425" s="96" t="n"/>
     </row>
     <row r="426" ht="16.5" customHeight="1">
       <c r="A426" s="95" t="n"/>
       <c r="B426" s="95" t="n"/>
       <c r="C426" s="95" t="n"/>
-      <c r="D426" s="91" t="inlineStr">
-        <is>
-          <t>港建*(3093)</t>
-        </is>
-      </c>
-      <c r="E426" s="92" t="n">
-        <v>150</v>
-      </c>
-      <c r="F426" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G426" s="92" t="n">
-        <v>929</v>
-      </c>
-      <c r="H426" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="I426" s="92" t="n">
-        <v>929</v>
-      </c>
-      <c r="J426" s="93" t="n">
-        <v>61.93</v>
-      </c>
-      <c r="K426" s="93" t="n">
-        <v>0</v>
-      </c>
-      <c r="L426" s="96">
-        <f>F426*(K426-J426)</f>
-        <v/>
-      </c>
+      <c r="D426" s="91" t="n"/>
+      <c r="E426" s="92" t="n"/>
+      <c r="F426" s="92" t="n"/>
+      <c r="G426" s="92" t="n"/>
+      <c r="H426" s="92" t="n"/>
+      <c r="I426" s="92" t="n"/>
+      <c r="J426" s="93" t="n"/>
+      <c r="K426" s="93" t="n"/>
+      <c r="L426" s="96" t="n"/>
     </row>
     <row r="427" ht="16.5" customHeight="1">
       <c r="A427" s="95" t="n"/>
       <c r="B427" s="95" t="n"/>
       <c r="C427" s="95" t="n"/>
-      <c r="D427" s="91" t="inlineStr">
-        <is>
-          <t>仁寶(2324)</t>
-        </is>
-      </c>
-      <c r="E427" s="92" t="n">
-        <v>184</v>
-      </c>
-      <c r="F427" s="92" t="n">
-        <v>68</v>
-      </c>
-      <c r="G427" s="92" t="n">
-        <v>762</v>
-      </c>
-      <c r="H427" s="92" t="n">
-        <v>282</v>
-      </c>
-      <c r="I427" s="92" t="n">
-        <v>480</v>
-      </c>
-      <c r="J427" s="93" t="n">
-        <v>41.4</v>
-      </c>
-      <c r="K427" s="93" t="n">
-        <v>41.4</v>
-      </c>
-      <c r="L427" s="96">
-        <f>F427*(K427-J427)</f>
-        <v/>
-      </c>
+      <c r="D427" s="91" t="n"/>
+      <c r="E427" s="92" t="n"/>
+      <c r="F427" s="92" t="n"/>
+      <c r="G427" s="92" t="n"/>
+      <c r="H427" s="92" t="n"/>
+      <c r="I427" s="92" t="n"/>
+      <c r="J427" s="93" t="n"/>
+      <c r="K427" s="93" t="n"/>
+      <c r="L427" s="96" t="n"/>
     </row>
     <row r="428" ht="16.5" customHeight="1">
       <c r="A428" s="95" t="n"/>
       <c r="B428" s="95" t="n"/>
       <c r="C428" s="95" t="n"/>
-      <c r="D428" s="91" t="inlineStr">
-        <is>
-          <t>大量(3167)</t>
-        </is>
-      </c>
-      <c r="E428" s="92" t="n">
-        <v>7</v>
-      </c>
-      <c r="F428" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G428" s="92" t="n">
-        <v>712</v>
-      </c>
-      <c r="H428" s="92" t="n">
-        <v>0</v>
-      </c>
-      <c r="I428" s="92" t="n">
-        <v>712</v>
-      </c>
-      <c r="J428" s="93" t="n">
-        <v>1017.14</v>
-      </c>
-      <c r="K428" s="93" t="n">
-        <v>0</v>
-      </c>
-      <c r="L428" s="96">
-        <f>F428*(K428-J428)</f>
-        <v/>
-      </c>
+      <c r="D428" s="91" t="n"/>
+      <c r="E428" s="92" t="n"/>
+      <c r="F428" s="92" t="n"/>
+      <c r="G428" s="92" t="n"/>
+      <c r="H428" s="92" t="n"/>
+      <c r="I428" s="92" t="n"/>
+      <c r="J428" s="93" t="n"/>
+      <c r="K428" s="93" t="n"/>
+      <c r="L428" s="96" t="n"/>
     </row>
     <row r="429" ht="16.5" customHeight="1">
       <c r="A429" s="95" t="n"/>
       <c r="B429" s="95" t="n"/>
       <c r="C429" s="95" t="n"/>
-      <c r="D429" s="91" t="inlineStr">
-        <is>
-          <t>新纖(1409)</t>
-        </is>
-      </c>
-      <c r="E429" s="92" t="n">
-        <v>106</v>
-      </c>
-      <c r="F429" s="92" t="n">
-        <v>51</v>
-      </c>
-      <c r="G429" s="92" t="n">
-        <v>277</v>
-      </c>
-      <c r="H429" s="92" t="n">
-        <v>133</v>
-      </c>
-      <c r="I429" s="92" t="n">
-        <v>144</v>
-      </c>
-      <c r="J429" s="93" t="n">
-        <v>26.15</v>
-      </c>
-      <c r="K429" s="93" t="n">
-        <v>26.16</v>
-      </c>
-      <c r="L429" s="96">
-        <f>F429*(K429-J429)</f>
-        <v/>
-      </c>
+      <c r="D429" s="91" t="n"/>
+      <c r="E429" s="92" t="n"/>
+      <c r="F429" s="92" t="n"/>
+      <c r="G429" s="92" t="n"/>
+      <c r="H429" s="92" t="n"/>
+      <c r="I429" s="92" t="n"/>
+      <c r="J429" s="93" t="n"/>
+      <c r="K429" s="93" t="n"/>
+      <c r="L429" s="96" t="n"/>
     </row>
     <row r="430" ht="16.5" customHeight="1">
       <c r="A430" s="99" t="inlineStr">

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-06-06 14:14
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-06.xlsx
+++ b/data/reports/chip_radar_2026-06.xlsx
@@ -8065,10 +8065,10 @@
         </is>
       </c>
       <c r="E189" s="31" t="n">
-        <v>1776</v>
+        <v>1771</v>
       </c>
       <c r="F189" s="31" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G189" s="31" t="n">
         <v>23292</v>
@@ -8080,12 +8080,12 @@
         <v>21855</v>
       </c>
       <c r="J189" s="32" t="n">
-        <v>131.15</v>
+        <v>131.52</v>
       </c>
       <c r="K189" s="32" t="n">
-        <v>130.67</v>
-      </c>
-      <c r="L189" s="33">
+        <v>131.87</v>
+      </c>
+      <c r="L189" s="35">
         <f>F189*(K189-J189)</f>
         <v/>
       </c>
@@ -8135,10 +8135,10 @@
         </is>
       </c>
       <c r="E191" s="31" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F191" s="31" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G191" s="31" t="n">
         <v>5757</v>
@@ -8150,12 +8150,12 @@
         <v>4744</v>
       </c>
       <c r="J191" s="32" t="n">
-        <v>738.05</v>
+        <v>767.5700000000001</v>
       </c>
       <c r="K191" s="32" t="n">
-        <v>723.5</v>
-      </c>
-      <c r="L191" s="33">
+        <v>779.15</v>
+      </c>
+      <c r="L191" s="35">
         <f>F191*(K191-J191)</f>
         <v/>
       </c>
@@ -8170,10 +8170,10 @@
         </is>
       </c>
       <c r="E192" s="31" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F192" s="31" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G192" s="31" t="n">
         <v>4738</v>
@@ -8185,12 +8185,12 @@
         <v>2441</v>
       </c>
       <c r="J192" s="32" t="n">
-        <v>361.64</v>
+        <v>358.9</v>
       </c>
       <c r="K192" s="32" t="n">
-        <v>364.59</v>
-      </c>
-      <c r="L192" s="35">
+        <v>358.89</v>
+      </c>
+      <c r="L192" s="33">
         <f>F192*(K192-J192)</f>
         <v/>
       </c>
@@ -8205,7 +8205,7 @@
         </is>
       </c>
       <c r="E193" s="31" t="n">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="F193" s="31" t="n">
         <v>23</v>
@@ -8220,12 +8220,12 @@
         <v>3857</v>
       </c>
       <c r="J193" s="32" t="n">
-        <v>140.27</v>
+        <v>141.7</v>
       </c>
       <c r="K193" s="32" t="n">
         <v>140.39</v>
       </c>
-      <c r="L193" s="35">
+      <c r="L193" s="33">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -8306,29 +8306,29 @@
       <c r="C196" s="34" t="n"/>
       <c r="D196" s="30" t="inlineStr">
         <is>
-          <t>友達(2409)</t>
+          <t>大綜(3147)</t>
         </is>
       </c>
       <c r="E196" s="31" t="n">
-        <v>1046</v>
+        <v>106</v>
       </c>
       <c r="F196" s="31" t="n">
-        <v>943</v>
+        <v>0</v>
       </c>
       <c r="G196" s="31" t="n">
-        <v>2835</v>
+        <v>3016</v>
       </c>
       <c r="H196" s="31" t="n">
-        <v>2556</v>
+        <v>0</v>
       </c>
       <c r="I196" s="31" t="n">
-        <v>279</v>
+        <v>3016</v>
       </c>
       <c r="J196" s="32" t="n">
-        <v>27.1</v>
+        <v>284.5</v>
       </c>
       <c r="K196" s="32" t="n">
-        <v>27.1</v>
+        <v>0</v>
       </c>
       <c r="L196" s="35">
         <f>F196*(K196-J196)</f>
@@ -8376,31 +8376,31 @@
       <c r="C198" s="34" t="n"/>
       <c r="D198" s="30" t="inlineStr">
         <is>
-          <t>群創(3481)</t>
+          <t>華邦電(2344)</t>
         </is>
       </c>
       <c r="E198" s="31" t="n">
-        <v>442</v>
+        <v>158</v>
       </c>
       <c r="F198" s="31" t="n">
-        <v>320</v>
+        <v>47</v>
       </c>
       <c r="G198" s="31" t="n">
-        <v>2305</v>
+        <v>2560</v>
       </c>
       <c r="H198" s="31" t="n">
-        <v>1643</v>
+        <v>761</v>
       </c>
       <c r="I198" s="31" t="n">
-        <v>662</v>
+        <v>1799</v>
       </c>
       <c r="J198" s="32" t="n">
-        <v>52.15</v>
+        <v>162</v>
       </c>
       <c r="K198" s="32" t="n">
-        <v>51.35</v>
-      </c>
-      <c r="L198" s="33">
+        <v>162</v>
+      </c>
+      <c r="L198" s="35">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>

</xml_diff>